<commit_message>
Edit cards; continue refining code
</commit_message>
<xml_diff>
--- a/Cards.xlsx
+++ b/Cards.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wk725/Documents/Randomness/Custom_Board_Games/The_Ultimate_Storm_Pacific_V2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wk725/Documents/Randomness/Custom_Board_Games/The_Ultimate_Storm/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBEBE595-9180-C943-8751-D1514A2E82E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E43A3F80-C5A6-9342-B0AB-4BC8FA2A16DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11340" yWindow="1080" windowWidth="16660" windowHeight="16540" xr2:uid="{FB1CF6F0-4410-014C-ADA4-54BAFA659877}"/>
+    <workbookView xWindow="11340" yWindow="1080" windowWidth="15840" windowHeight="16540" xr2:uid="{FB1CF6F0-4410-014C-ADA4-54BAFA659877}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -170,9 +170,6 @@
     <t>Stop one opponent of your choice from intensifying for 3 rounds</t>
   </si>
   <si>
-    <t>Protect one city of your choice from being impacted for 3 rounds</t>
-  </si>
-  <si>
     <t>Impact one city of your choice at an adjacent grid box</t>
   </si>
   <si>
@@ -203,21 +200,12 @@
     <t>Move in the opposite direction of a movement card</t>
   </si>
   <si>
-    <t>Random Teleportation</t>
-  </si>
-  <si>
     <t>Survival of the Fittest</t>
   </si>
   <si>
-    <t>Become immune to any weakening for the next 3 rounds</t>
-  </si>
-  <si>
     <t>Factory Reset</t>
   </si>
   <si>
-    <t>Fortune Teller</t>
-  </si>
-  <si>
     <t>W 4</t>
   </si>
   <si>
@@ -263,16 +251,28 @@
     <t>Discard all your current cards and take 10 new cards from the deck</t>
   </si>
   <si>
-    <t>Roll the dice and teleport to that genesis point</t>
-  </si>
-  <si>
-    <t>Take a look at the next 5 cards in the deck, pick one to keep</t>
-  </si>
-  <si>
     <t>W 1 S 2</t>
   </si>
   <si>
     <t>W 1 N 3</t>
+  </si>
+  <si>
+    <t>Breaking Free</t>
+  </si>
+  <si>
+    <t>Become immune from any weakening for the next 3 rounds</t>
+  </si>
+  <si>
+    <t>Protect one city of your choice from being impacted by any opponent for 3 rounds</t>
+  </si>
+  <si>
+    <t>Remove all negative effects affecting yourself</t>
+  </si>
+  <si>
+    <t>Instant Teleportation</t>
+  </si>
+  <si>
+    <t>Teleport to a genesis point of your choice</t>
   </si>
 </sst>
 </file>
@@ -654,7 +654,7 @@
         <v>4</v>
       </c>
       <c r="C2">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -665,7 +665,7 @@
         <v>5</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -676,7 +676,7 @@
         <v>12</v>
       </c>
       <c r="C4">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -684,10 +684,10 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -695,7 +695,7 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -720,7 +720,7 @@
         <v>10</v>
       </c>
       <c r="C8">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -742,7 +742,7 @@
         <v>6</v>
       </c>
       <c r="C10">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
@@ -753,7 +753,7 @@
         <v>9</v>
       </c>
       <c r="C11">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
@@ -764,7 +764,7 @@
         <v>13</v>
       </c>
       <c r="C12">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
@@ -772,10 +772,10 @@
         <v>1</v>
       </c>
       <c r="B13" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
@@ -783,7 +783,7 @@
         <v>1</v>
       </c>
       <c r="B14" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -797,7 +797,7 @@
         <v>7</v>
       </c>
       <c r="C15">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
@@ -808,7 +808,7 @@
         <v>11</v>
       </c>
       <c r="C16">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
@@ -816,7 +816,7 @@
         <v>1</v>
       </c>
       <c r="B17" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C17">
         <v>1</v>
@@ -841,7 +841,7 @@
         <v>34</v>
       </c>
       <c r="C19">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
@@ -882,7 +882,7 @@
         <v>1</v>
       </c>
       <c r="B23" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="C23">
         <v>1</v>
@@ -896,7 +896,7 @@
         <v>17</v>
       </c>
       <c r="C24">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
@@ -907,7 +907,7 @@
         <v>38</v>
       </c>
       <c r="C25">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
@@ -915,7 +915,7 @@
         <v>1</v>
       </c>
       <c r="B26" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C26">
         <v>1</v>
@@ -940,7 +940,7 @@
         <v>16</v>
       </c>
       <c r="C28">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
@@ -951,7 +951,7 @@
         <v>36</v>
       </c>
       <c r="C29">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
@@ -1003,13 +1003,13 @@
         <v>1</v>
       </c>
       <c r="B34" t="s">
+        <v>61</v>
+      </c>
+      <c r="C34">
+        <v>4</v>
+      </c>
+      <c r="D34" t="s">
         <v>65</v>
-      </c>
-      <c r="C34">
-        <v>2</v>
-      </c>
-      <c r="D34" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
@@ -1017,13 +1017,13 @@
         <v>1</v>
       </c>
       <c r="B35" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C35">
         <v>2</v>
       </c>
       <c r="D35" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
@@ -1031,13 +1031,13 @@
         <v>1</v>
       </c>
       <c r="B36" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D36" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
@@ -1045,13 +1045,13 @@
         <v>1</v>
       </c>
       <c r="B37" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C37">
         <v>1</v>
       </c>
       <c r="D37" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
@@ -1059,10 +1059,10 @@
         <v>1</v>
       </c>
       <c r="B38" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C38">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
@@ -1070,10 +1070,10 @@
         <v>1</v>
       </c>
       <c r="B39" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C39">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
@@ -1081,14 +1081,14 @@
         <v>1</v>
       </c>
       <c r="B40" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C40">
         <v>2</v>
       </c>
       <c r="E40">
         <f>SUM(C2:C40)</f>
-        <v>75</v>
+        <v>100</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
@@ -1099,7 +1099,7 @@
         <v>30</v>
       </c>
       <c r="C41">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
@@ -1110,7 +1110,7 @@
         <v>31</v>
       </c>
       <c r="C42">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
@@ -1121,7 +1121,7 @@
         <v>32</v>
       </c>
       <c r="C43">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
@@ -1132,7 +1132,7 @@
         <v>33</v>
       </c>
       <c r="C44">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
@@ -1143,7 +1143,7 @@
         <v>41</v>
       </c>
       <c r="C45">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
@@ -1154,7 +1154,7 @@
         <v>42</v>
       </c>
       <c r="C46">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
@@ -1162,17 +1162,17 @@
         <v>19</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C47">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D47" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="E47">
         <f>SUM(C41:C47)</f>
-        <v>75</v>
+        <v>100</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
@@ -1183,10 +1183,10 @@
         <v>21</v>
       </c>
       <c r="C48">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D48" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
@@ -1194,13 +1194,13 @@
         <v>20</v>
       </c>
       <c r="B49" t="s">
+        <v>46</v>
+      </c>
+      <c r="C49">
+        <v>10</v>
+      </c>
+      <c r="D49" t="s">
         <v>47</v>
-      </c>
-      <c r="C49">
-        <v>5</v>
-      </c>
-      <c r="D49" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
@@ -1208,13 +1208,13 @@
         <v>20</v>
       </c>
       <c r="B50" t="s">
+        <v>52</v>
+      </c>
+      <c r="C50">
+        <v>5</v>
+      </c>
+      <c r="D50" t="s">
         <v>53</v>
-      </c>
-      <c r="C50">
-        <v>2</v>
-      </c>
-      <c r="D50" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
@@ -1222,13 +1222,13 @@
         <v>20</v>
       </c>
       <c r="B51" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C51">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D51" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.2">
@@ -1264,13 +1264,13 @@
         <v>20</v>
       </c>
       <c r="B54" t="s">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="C54">
         <v>2</v>
       </c>
       <c r="D54" t="s">
-        <v>45</v>
+        <v>75</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.2">
@@ -1278,7 +1278,7 @@
         <v>20</v>
       </c>
       <c r="B55" t="s">
-        <v>49</v>
+        <v>25</v>
       </c>
       <c r="C55">
         <v>2</v>
@@ -1292,13 +1292,13 @@
         <v>20</v>
       </c>
       <c r="B56" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="C56">
         <v>2</v>
       </c>
       <c r="D56" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.2">
@@ -1306,13 +1306,13 @@
         <v>20</v>
       </c>
       <c r="B57" t="s">
-        <v>58</v>
+        <v>77</v>
       </c>
       <c r="C57">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D57" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.2">
@@ -1320,13 +1320,13 @@
         <v>20</v>
       </c>
       <c r="B58" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C58">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D58" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.2">
@@ -1334,17 +1334,17 @@
         <v>20</v>
       </c>
       <c r="B59" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C59">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D59" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="E59">
         <f>SUM(C48:C59)</f>
-        <v>30</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updates to cards, rule book and code
</commit_message>
<xml_diff>
--- a/Cards.xlsx
+++ b/Cards.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wk725/Documents/Randomness/Custom_Board_Games/The_Ultimate_Storm/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E43A3F80-C5A6-9342-B0AB-4BC8FA2A16DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D75E517-DCA9-E14C-AD23-4DDB2F617429}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11340" yWindow="1080" windowWidth="15840" windowHeight="16540" xr2:uid="{FB1CF6F0-4410-014C-ADA4-54BAFA659877}"/>
+    <workbookView xWindow="13140" yWindow="1040" windowWidth="15840" windowHeight="16540" xr2:uid="{FB1CF6F0-4410-014C-ADA4-54BAFA659877}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -654,7 +654,7 @@
         <v>4</v>
       </c>
       <c r="C2">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -665,7 +665,7 @@
         <v>5</v>
       </c>
       <c r="C3">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -676,7 +676,7 @@
         <v>12</v>
       </c>
       <c r="C4">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -720,7 +720,7 @@
         <v>10</v>
       </c>
       <c r="C8">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -742,7 +742,7 @@
         <v>6</v>
       </c>
       <c r="C10">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
@@ -808,7 +808,7 @@
         <v>11</v>
       </c>
       <c r="C16">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
@@ -1006,7 +1006,7 @@
         <v>61</v>
       </c>
       <c r="C34">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D34" t="s">
         <v>65</v>
@@ -1048,7 +1048,7 @@
         <v>64</v>
       </c>
       <c r="C37">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D37" t="s">
         <v>65</v>
@@ -1197,7 +1197,7 @@
         <v>46</v>
       </c>
       <c r="C49">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D49" t="s">
         <v>47</v>
@@ -1211,7 +1211,7 @@
         <v>52</v>
       </c>
       <c r="C50">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D50" t="s">
         <v>53</v>
@@ -1222,13 +1222,13 @@
         <v>20</v>
       </c>
       <c r="B51" t="s">
-        <v>54</v>
+        <v>77</v>
       </c>
       <c r="C51">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D51" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.2">
@@ -1236,13 +1236,13 @@
         <v>20</v>
       </c>
       <c r="B52" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
       <c r="C52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D52" t="s">
-        <v>43</v>
+        <v>74</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
@@ -1250,13 +1250,13 @@
         <v>20</v>
       </c>
       <c r="B53" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C53">
         <v>2</v>
       </c>
       <c r="D53" t="s">
-        <v>26</v>
+        <v>43</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.2">
@@ -1264,13 +1264,13 @@
         <v>20</v>
       </c>
       <c r="B54" t="s">
-        <v>48</v>
+        <v>23</v>
       </c>
       <c r="C54">
         <v>2</v>
       </c>
       <c r="D54" t="s">
-        <v>75</v>
+        <v>26</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.2">
@@ -1278,13 +1278,13 @@
         <v>20</v>
       </c>
       <c r="B55" t="s">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="C55">
         <v>2</v>
       </c>
       <c r="D55" t="s">
-        <v>44</v>
+        <v>75</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.2">
@@ -1292,13 +1292,13 @@
         <v>20</v>
       </c>
       <c r="B56" t="s">
-        <v>73</v>
+        <v>25</v>
       </c>
       <c r="C56">
         <v>2</v>
       </c>
       <c r="D56" t="s">
-        <v>76</v>
+        <v>44</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.2">
@@ -1306,13 +1306,13 @@
         <v>20</v>
       </c>
       <c r="B57" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C57">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D57" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.2">
@@ -1323,7 +1323,7 @@
         <v>68</v>
       </c>
       <c r="C58">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D58" t="s">
         <v>69</v>
@@ -1337,7 +1337,7 @@
         <v>55</v>
       </c>
       <c r="C59">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D59" t="s">
         <v>70</v>

</xml_diff>